<commit_message>
Re-run audit pass: update SPINS_CSV path and regenerate workbook
Co-authored-by: FarPointer <47090086+FarPointer@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/shows/convergence-zone/playlists/analysis/cz-playlist-spinitron-audit.xlsx
+++ b/shows/convergence-zone/playlists/analysis/cz-playlist-spinitron-audit.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$4:$M$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Add to Spinitron'!$A$4:$M$67</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Check metadata'!$A$4:$K$93</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spins not in notes'!$A$4:$H$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Spins not in notes'!$A$4:$H$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Method'!$A$4:$B$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1222,7 +1222,7 @@
         <v>22</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H16" s="8" t="n">
         <v>20</v>
@@ -1231,11 +1231,11 @@
         <v>2</v>
       </c>
       <c r="J16" s="8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="L16" s="8" t="inlineStr">
@@ -10046,7 +10046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11215,27 +11215,27 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>8:32 pm</t>
+          <t>10:07 pm</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Sea Lemon</t>
+          <t>Talkdemonic</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>In The Flowers</t>
+          <t>Early and Forever</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Diving For A Prize</t>
+          <t>Early and Forever</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Luminelle Recordings</t>
+          <t>Bathysphere Records</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
@@ -11249,50 +11249,8 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>2025-09-09</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>10:07 pm</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Talkdemonic</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Early and Forever</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Early and Forever</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>Bathysphere Records</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>not in the note - worth a look</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>both lists agree closely - little to do</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:H32"/>
+  <autoFilter ref="A4:H31"/>
   <mergeCells count="1">
     <mergeCell ref="A2:H2"/>
   </mergeCells>
@@ -11431,7 +11389,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Spins-search-results-12-5-19-8-4-26-for-KSER.csv - 3,282 spins across 164 playlists, 2023-05-30 to 2026-07-28.</t>
+          <t>Spins-search-results-12-10-19-8-9-26-for-KSER.csv - 3,432 spins across 165 broadcast dates, 2023-05-30 to 2026-08-04.</t>
         </is>
       </c>
     </row>
@@ -11443,7 +11401,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>12 of 164 Spinitron playlists - the ones with a matching set list. The rest have neither a published playlist nor a usable prep note.</t>
+          <t>12 of 165 Spinitron broadcast dates - the ones with a matching set list. The rest have neither a published playlist nor a usable prep note.</t>
         </is>
       </c>
     </row>
@@ -11455,7 +11413,7 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>67 of 83 OneNote files are promo blurbs with no track listing. 39 of 66 site posts are promo prose with no playlist table. Four published playlists never matched any Spinitron broadcast (episodes 003, 009, 010, 011): they aired before Spinitron logging began on 2023-05-30 and were never replayed.</t>
+          <t>71 of 83 OneNote files are promo blurbs with no track listing. The site scrape did not run, so none of the 47 archived convergencezone.fm playlists were used - every audited broadcast fell back to its OneNote note.</t>
         </is>
       </c>
     </row>

</xml_diff>